<commit_message>
Started work on sas-06-05
</commit_message>
<xml_diff>
--- a/06/data/merge-types.xlsx
+++ b/06/data/merge-types.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve\git\5507-2025b\06\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F24C78-9944-4D00-8ACE-F1E44EB21E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D40F11-F4D8-4E3A-9919-EDE5845F9DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{3B3174C3-09F6-4A66-8032-021BCA7D1A92}"/>
+    <workbookView xWindow="-28920" yWindow="-1695" windowWidth="29040" windowHeight="17520" xr2:uid="{3B3174C3-09F6-4A66-8032-021BCA7D1A92}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -304,25 +304,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
@@ -662,7 +661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4437E6BB-E90B-4BD2-BD79-42E7B90A3E39}">
-  <dimension ref="B2:R102"/>
+  <dimension ref="B2:M101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="1"/>
@@ -675,7 +674,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -695,319 +694,225 @@
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" s="5"/>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L5" s="6"/>
-      <c r="M5" s="7"/>
+      <c r="M5" s="6"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="5"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="7"/>
+      <c r="M6" s="6"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="11" t="s">
+      <c r="C7" s="9"/>
+      <c r="D7" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10" t="s">
+      <c r="E7" s="9"/>
+      <c r="F7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="G7" s="10"/>
-      <c r="H7" s="11" t="s">
+      <c r="G7" s="9"/>
+      <c r="H7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="6"/>
-      <c r="J7" s="10" t="s">
+      <c r="J7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="K7" s="10"/>
-      <c r="L7" s="6" t="s">
+      <c r="K7" s="9"/>
+      <c r="L7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="M7" s="7"/>
+      <c r="M7" s="6"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="5">
         <v>1001</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6">
+      <c r="F8" s="1">
         <v>1001</v>
       </c>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6">
+      <c r="J8" s="1">
         <v>1001</v>
       </c>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6" t="s">
+      <c r="L8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M8" s="7"/>
+      <c r="M8" s="6"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="5">
         <v>1002</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6">
+      <c r="F9" s="1">
         <v>1003</v>
       </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6">
+      <c r="J9" s="1">
         <v>1002</v>
       </c>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6" t="s">
+      <c r="L9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="M9" s="7"/>
+      <c r="M9" s="6"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" s="5">
         <v>1006</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6">
+      <c r="F10" s="1">
         <v>1005</v>
       </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6">
+      <c r="J10" s="1">
         <v>1003</v>
       </c>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6" t="s">
+      <c r="L10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="M10" s="7"/>
+      <c r="M10" s="6"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11" s="5">
         <v>1007</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6">
+      <c r="F11" s="1">
         <v>1006</v>
       </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6">
+      <c r="J11" s="1">
         <v>1005</v>
       </c>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6" t="s">
+      <c r="L11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="M11" s="7"/>
+      <c r="M11" s="6"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="5">
         <v>1008</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6">
+      <c r="F12" s="1">
         <v>1008</v>
       </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6">
+      <c r="J12" s="1">
         <v>1006</v>
       </c>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6" t="s">
+      <c r="L12" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M12" s="7"/>
+      <c r="M12" s="6"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="10" t="s">
+      <c r="C13" s="9"/>
+      <c r="F13" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G13" s="10"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6">
+      <c r="G13" s="9"/>
+      <c r="J13" s="1">
         <v>1007</v>
       </c>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6" t="s">
+      <c r="L13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="M13" s="7"/>
+      <c r="M13" s="6"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="5">
         <v>1098</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6">
+      <c r="F14" s="1">
         <v>1098</v>
       </c>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6" t="s">
+      <c r="H14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6">
+      <c r="J14" s="1">
         <v>1008</v>
       </c>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6" t="s">
+      <c r="L14" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M14" s="7"/>
+      <c r="M14" s="6"/>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B15" s="5"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="10" t="s">
+      <c r="J15" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="K15" s="10"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="7"/>
+      <c r="K15" s="9"/>
+      <c r="M15" s="6"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" s="5"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6">
+      <c r="J16" s="1">
         <v>1098</v>
       </c>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6" t="s">
+      <c r="L16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M16" s="7"/>
+      <c r="M16" s="6"/>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B17" s="12"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="14"/>
-    </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="13"/>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B21" s="2"/>
@@ -1025,429 +930,304 @@
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B22" s="5"/>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="8" t="s">
+      <c r="G22" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="8" t="s">
+      <c r="K22" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L22" s="6"/>
-      <c r="M22" s="7"/>
+      <c r="M22" s="6"/>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B23" s="5"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="6"/>
-      <c r="M23" s="7"/>
+      <c r="M23" s="6"/>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11" t="s">
+      <c r="C24" s="9"/>
+      <c r="D24" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10" t="s">
+      <c r="E24" s="9"/>
+      <c r="F24" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="G24" s="10"/>
-      <c r="H24" s="11" t="s">
+      <c r="G24" s="9"/>
+      <c r="H24" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="I24" s="6"/>
-      <c r="J24" s="10" t="s">
+      <c r="J24" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="K24" s="10"/>
-      <c r="L24" s="6" t="s">
+      <c r="K24" s="9"/>
+      <c r="L24" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="M24" s="7"/>
+      <c r="M24" s="6"/>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B25" s="5">
         <v>1001</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6">
+      <c r="F25" s="1">
         <v>1001</v>
       </c>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6" t="s">
+      <c r="H25" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6">
+      <c r="J25" s="1">
         <v>1001</v>
       </c>
-      <c r="K25" s="6"/>
-      <c r="L25" s="6" t="s">
+      <c r="L25" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M25" s="7"/>
+      <c r="M25" s="6"/>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B26" s="5">
         <v>1002</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6">
+      <c r="F26" s="1">
         <v>1001</v>
       </c>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6" t="s">
+      <c r="H26" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6">
+      <c r="J26" s="1">
         <v>1001</v>
       </c>
-      <c r="K26" s="6"/>
-      <c r="L26" s="6" t="s">
+      <c r="L26" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M26" s="7"/>
+      <c r="M26" s="6"/>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B27" s="5">
         <v>1004</v>
       </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6">
+      <c r="F27" s="1">
         <v>1001</v>
       </c>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6" t="s">
+      <c r="H27" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6">
+      <c r="J27" s="1">
         <v>1001</v>
       </c>
-      <c r="K27" s="6"/>
-      <c r="L27" s="6" t="s">
+      <c r="L27" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="M27" s="7"/>
+      <c r="M27" s="6"/>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B28" s="5">
         <v>1005</v>
       </c>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6">
+      <c r="F28" s="1">
         <v>1002</v>
       </c>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6" t="s">
+      <c r="H28" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I28" s="6"/>
-      <c r="J28" s="6">
+      <c r="J28" s="1">
         <v>1002</v>
       </c>
-      <c r="K28" s="6"/>
-      <c r="L28" s="6" t="s">
+      <c r="L28" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="M28" s="7"/>
+      <c r="M28" s="6"/>
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B29" s="5">
         <v>1006</v>
       </c>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6">
+      <c r="F29" s="1">
         <v>1002</v>
       </c>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6" t="s">
+      <c r="H29" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I29" s="6"/>
-      <c r="J29" s="6">
+      <c r="J29" s="1">
         <v>1002</v>
       </c>
-      <c r="K29" s="6"/>
-      <c r="L29" s="6" t="s">
+      <c r="L29" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M29" s="7"/>
+      <c r="M29" s="6"/>
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C30" s="10"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6">
+      <c r="C30" s="9"/>
+      <c r="F30" s="1">
         <v>1003</v>
       </c>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6" t="s">
+      <c r="H30" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6">
+      <c r="J30" s="1">
         <v>1003</v>
       </c>
-      <c r="K30" s="6"/>
-      <c r="L30" s="6" t="s">
+      <c r="L30" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="M30" s="7"/>
+      <c r="M30" s="6"/>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B31" s="5">
         <v>1098</v>
       </c>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6">
+      <c r="F31" s="1">
         <v>1006</v>
       </c>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6" t="s">
+      <c r="H31" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="I31" s="6"/>
-      <c r="J31" s="6">
+      <c r="J31" s="1">
         <v>1004</v>
       </c>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6" t="s">
+      <c r="L31" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M31" s="7"/>
+      <c r="M31" s="6"/>
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B32" s="5"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6">
+      <c r="F32" s="1">
         <v>1006</v>
       </c>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6" t="s">
+      <c r="H32" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="I32" s="6"/>
-      <c r="J32" s="6">
+      <c r="J32" s="1">
         <v>1005</v>
       </c>
-      <c r="K32" s="6"/>
-      <c r="L32" s="11" t="s">
+      <c r="L32" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="M32" s="7"/>
+      <c r="M32" s="6"/>
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B33" s="5"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6">
+      <c r="F33" s="1">
         <v>1006</v>
       </c>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6" t="s">
+      <c r="H33" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6">
+      <c r="J33" s="1">
         <v>1006</v>
       </c>
-      <c r="K33" s="6"/>
-      <c r="L33" s="6" t="s">
+      <c r="L33" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M33" s="7"/>
+      <c r="M33" s="6"/>
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B34" s="5"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="10" t="s">
+      <c r="F34" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G34" s="10"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6">
+      <c r="G34" s="9"/>
+      <c r="J34" s="1">
         <v>1006</v>
       </c>
-      <c r="K34" s="6"/>
-      <c r="L34" s="6" t="s">
+      <c r="L34" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="M34" s="7"/>
+      <c r="M34" s="6"/>
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B35" s="5"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6">
+      <c r="F35" s="1">
         <v>1098</v>
       </c>
-      <c r="G35" s="6"/>
-      <c r="H35" s="6" t="s">
+      <c r="H35" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6">
+      <c r="J35" s="1">
         <v>1006</v>
       </c>
-      <c r="K35" s="6"/>
-      <c r="L35" s="6" t="s">
+      <c r="L35" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="M35" s="7"/>
+      <c r="M35" s="6"/>
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B36" s="5"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6">
+      <c r="F36" s="1">
         <v>1098</v>
       </c>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6" t="s">
+      <c r="H36" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="I36" s="6"/>
-      <c r="J36" s="10" t="s">
+      <c r="J36" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="7"/>
+      <c r="M36" s="6"/>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B37" s="5"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6">
+      <c r="J37" s="1">
         <v>1098</v>
       </c>
-      <c r="K37" s="6"/>
-      <c r="L37" s="6" t="s">
+      <c r="L37" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M37" s="7"/>
+      <c r="M37" s="6"/>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B38" s="5"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
-      <c r="E38" s="6"/>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-      <c r="H38" s="6"/>
-      <c r="I38" s="6"/>
-      <c r="J38" s="6">
+      <c r="J38" s="1">
         <v>1098</v>
       </c>
-      <c r="K38" s="6"/>
-      <c r="L38" s="6" t="s">
+      <c r="L38" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="M38" s="7"/>
+      <c r="M38" s="6"/>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B39" s="12"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="13"/>
-      <c r="J39" s="13"/>
-      <c r="K39" s="13"/>
-      <c r="L39" s="13"/>
-      <c r="M39" s="14"/>
-    </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B40" s="6"/>
-      <c r="C40" s="6"/>
-      <c r="D40" s="6"/>
-      <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
-      <c r="H40" s="6"/>
-      <c r="I40" s="6"/>
-      <c r="J40" s="6"/>
-      <c r="K40" s="6"/>
-      <c r="L40" s="6"/>
-      <c r="M40" s="6"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="12"/>
+      <c r="I39" s="12"/>
+      <c r="J39" s="12"/>
+      <c r="K39" s="12"/>
+      <c r="L39" s="12"/>
+      <c r="M39" s="13"/>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B41" s="6"/>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="6"/>
-      <c r="F41" s="6" t="s">
+      <c r="F41" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G41" s="6"/>
-      <c r="H41" s="6"/>
-      <c r="I41" s="6"/>
-      <c r="J41" s="6"/>
-      <c r="K41" s="6"/>
-      <c r="L41" s="6"/>
-      <c r="M41" s="6"/>
     </row>
     <row r="43" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B43" s="2"/>
@@ -1465,255 +1245,195 @@
     </row>
     <row r="44" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B44" s="5"/>
-      <c r="C44" s="8" t="s">
+      <c r="C44" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D44" s="6"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="6"/>
-      <c r="G44" s="8" t="s">
+      <c r="G44" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H44" s="6"/>
-      <c r="I44" s="6"/>
-      <c r="J44" s="6"/>
-      <c r="K44" s="8" t="s">
+      <c r="K44" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L44" s="6"/>
-      <c r="M44" s="7"/>
+      <c r="M44" s="6"/>
     </row>
     <row r="45" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B45" s="5"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="6"/>
-      <c r="G45" s="6"/>
-      <c r="H45" s="6"/>
-      <c r="I45" s="6"/>
-      <c r="J45" s="6"/>
-      <c r="K45" s="6"/>
-      <c r="L45" s="6"/>
-      <c r="M45" s="7"/>
+      <c r="M45" s="6"/>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B46" s="9" t="s">
+      <c r="B46" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C46" s="10"/>
-      <c r="D46" s="11" t="s">
+      <c r="C46" s="9"/>
+      <c r="D46" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E46" s="10"/>
-      <c r="F46" s="10" t="s">
+      <c r="E46" s="9"/>
+      <c r="F46" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="G46" s="10"/>
-      <c r="H46" s="11" t="s">
+      <c r="G46" s="9"/>
+      <c r="H46" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="I46" s="6"/>
-      <c r="J46" s="10" t="s">
+      <c r="J46" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="K46" s="10"/>
-      <c r="L46" s="6" t="s">
+      <c r="K46" s="9"/>
+      <c r="L46" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="M46" s="7"/>
+      <c r="M46" s="6"/>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B47" s="5">
         <v>1001</v>
       </c>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6" t="s">
+      <c r="D47" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E47" s="6"/>
-      <c r="F47" s="6">
+      <c r="F47" s="1">
         <v>1001</v>
       </c>
-      <c r="G47" s="6"/>
-      <c r="H47" s="6" t="s">
+      <c r="H47" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I47" s="6"/>
-      <c r="J47" s="6">
+      <c r="J47" s="1">
         <v>1001</v>
       </c>
-      <c r="K47" s="6"/>
-      <c r="L47" s="6" t="s">
+      <c r="L47" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M47" s="7"/>
+      <c r="M47" s="6"/>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B48" s="5">
         <v>1002</v>
       </c>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6" t="s">
+      <c r="D48" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E48" s="6"/>
-      <c r="F48" s="6">
+      <c r="F48" s="1">
         <v>1003</v>
       </c>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6" t="s">
+      <c r="H48" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I48" s="6"/>
-      <c r="J48" s="6">
+      <c r="J48" s="1">
         <v>1006</v>
       </c>
-      <c r="K48" s="6"/>
-      <c r="L48" s="6" t="s">
+      <c r="L48" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M48" s="7"/>
-    </row>
-    <row r="49" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="M48" s="6"/>
+    </row>
+    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B49" s="5">
         <v>1006</v>
       </c>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6" t="s">
+      <c r="D49" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E49" s="6"/>
-      <c r="F49" s="6">
+      <c r="F49" s="1">
         <v>1005</v>
       </c>
-      <c r="G49" s="6"/>
-      <c r="H49" s="6" t="s">
+      <c r="H49" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I49" s="6"/>
-      <c r="J49" s="6">
+      <c r="J49" s="1">
         <v>1008</v>
       </c>
-      <c r="K49" s="6"/>
-      <c r="L49" s="6" t="s">
+      <c r="L49" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M49" s="7"/>
-    </row>
-    <row r="50" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="M49" s="6"/>
+    </row>
+    <row r="50" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B50" s="5">
         <v>1007</v>
       </c>
-      <c r="C50" s="6"/>
-      <c r="D50" s="6" t="s">
+      <c r="D50" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E50" s="6"/>
-      <c r="F50" s="6">
+      <c r="F50" s="1">
         <v>1006</v>
       </c>
-      <c r="G50" s="6"/>
-      <c r="H50" s="6" t="s">
+      <c r="H50" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I50" s="6"/>
-      <c r="J50" s="10" t="s">
+      <c r="J50" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="K50" s="10"/>
-      <c r="L50" s="6"/>
-      <c r="M50" s="7"/>
-    </row>
-    <row r="51" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="K50" s="9"/>
+      <c r="M50" s="6"/>
+    </row>
+    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B51" s="5">
         <v>1008</v>
       </c>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6" t="s">
+      <c r="D51" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6">
+      <c r="F51" s="1">
         <v>1008</v>
       </c>
-      <c r="G51" s="6"/>
-      <c r="H51" s="6" t="s">
+      <c r="H51" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I51" s="6"/>
-      <c r="J51" s="6">
+      <c r="J51" s="1">
         <v>1098</v>
       </c>
-      <c r="K51" s="6"/>
-      <c r="L51" s="6" t="s">
+      <c r="L51" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M51" s="7"/>
-    </row>
-    <row r="52" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B52" s="9" t="s">
+      <c r="M51" s="6"/>
+    </row>
+    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B52" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C52" s="10"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
-      <c r="F52" s="10" t="s">
+      <c r="C52" s="9"/>
+      <c r="F52" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G52" s="10"/>
-      <c r="H52" s="6"/>
-      <c r="I52" s="6"/>
-      <c r="J52" s="6"/>
-      <c r="K52" s="6"/>
-      <c r="L52" s="6"/>
-      <c r="M52" s="7"/>
-    </row>
-    <row r="53" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="G52" s="9"/>
+      <c r="M52" s="6"/>
+    </row>
+    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B53" s="5">
         <v>1098</v>
       </c>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6" t="s">
+      <c r="D53" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E53" s="6"/>
-      <c r="F53" s="6">
+      <c r="F53" s="1">
         <v>1098</v>
       </c>
-      <c r="G53" s="6"/>
-      <c r="H53" s="6" t="s">
+      <c r="H53" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I53" s="6"/>
-      <c r="J53" s="6"/>
-      <c r="K53" s="6"/>
-      <c r="L53" s="6"/>
-      <c r="M53" s="7"/>
-    </row>
-    <row r="54" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B54" s="12"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="13"/>
-      <c r="G54" s="13"/>
-      <c r="H54" s="13"/>
-      <c r="I54" s="13"/>
-      <c r="J54" s="13"/>
-      <c r="K54" s="13"/>
-      <c r="L54" s="13"/>
-      <c r="M54" s="14"/>
-    </row>
-    <row r="56" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="F56" s="6" t="s">
+      <c r="M53" s="6"/>
+    </row>
+    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B54" s="11"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="12"/>
+      <c r="E54" s="12"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="12"/>
+      <c r="H54" s="12"/>
+      <c r="I54" s="12"/>
+      <c r="J54" s="12"/>
+      <c r="K54" s="12"/>
+      <c r="L54" s="12"/>
+      <c r="M54" s="13"/>
+    </row>
+    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="F56" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="P56" s="6"/>
-      <c r="Q56" s="6"/>
-      <c r="R56" s="6"/>
-    </row>
-    <row r="58" spans="2:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B58" s="2"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
@@ -1727,258 +1447,205 @@
       <c r="L58" s="3"/>
       <c r="M58" s="4"/>
     </row>
-    <row r="59" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B59" s="5"/>
-      <c r="C59" s="8" t="s">
+      <c r="C59" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D59" s="6"/>
-      <c r="E59" s="6"/>
-      <c r="F59" s="6"/>
-      <c r="G59" s="8" t="s">
+      <c r="G59" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H59" s="6"/>
-      <c r="I59" s="6"/>
-      <c r="J59" s="6"/>
-      <c r="K59" s="8" t="s">
+      <c r="K59" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L59" s="6"/>
-      <c r="M59" s="7"/>
-    </row>
-    <row r="60" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="M59" s="6"/>
+    </row>
+    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B60" s="5"/>
-      <c r="C60" s="6"/>
-      <c r="D60" s="6"/>
-      <c r="E60" s="6"/>
-      <c r="F60" s="6"/>
-      <c r="G60" s="6"/>
-      <c r="H60" s="6"/>
-      <c r="I60" s="6"/>
-      <c r="J60" s="6"/>
-      <c r="K60" s="6"/>
-      <c r="L60" s="6"/>
-      <c r="M60" s="7"/>
-    </row>
-    <row r="61" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B61" s="9" t="s">
+      <c r="M60" s="6"/>
+    </row>
+    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B61" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C61" s="10"/>
-      <c r="D61" s="11" t="s">
+      <c r="C61" s="9"/>
+      <c r="D61" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E61" s="10"/>
-      <c r="F61" s="10" t="s">
+      <c r="E61" s="9"/>
+      <c r="F61" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="G61" s="10"/>
-      <c r="H61" s="11" t="s">
+      <c r="G61" s="9"/>
+      <c r="H61" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="I61" s="6"/>
-      <c r="J61" s="10" t="s">
+      <c r="J61" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="K61" s="10"/>
-      <c r="L61" s="6" t="s">
+      <c r="K61" s="9"/>
+      <c r="L61" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="M61" s="7"/>
-    </row>
-    <row r="62" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="M61" s="6"/>
+    </row>
+    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B62" s="5">
         <v>1001</v>
       </c>
-      <c r="C62" s="6"/>
-      <c r="D62" s="6" t="s">
+      <c r="D62" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E62" s="6"/>
-      <c r="F62" s="6">
+      <c r="F62" s="1">
         <v>1001</v>
       </c>
-      <c r="G62" s="6"/>
-      <c r="H62" s="6" t="s">
+      <c r="H62" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I62" s="6"/>
-      <c r="J62" s="6">
+      <c r="J62" s="1">
         <v>1001</v>
       </c>
-      <c r="K62" s="6"/>
-      <c r="L62" s="6" t="s">
+      <c r="L62" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M62" s="7"/>
-    </row>
-    <row r="63" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="M62" s="6"/>
+    </row>
+    <row r="63" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B63" s="5">
         <v>1002</v>
       </c>
-      <c r="C63" s="6"/>
-      <c r="D63" s="6" t="s">
+      <c r="D63" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E63" s="6"/>
-      <c r="F63" s="6">
+      <c r="F63" s="1">
         <v>1003</v>
       </c>
-      <c r="G63" s="6"/>
-      <c r="H63" s="6" t="s">
+      <c r="H63" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I63" s="6"/>
-      <c r="J63" s="6">
+      <c r="J63" s="1">
         <v>1002</v>
       </c>
-      <c r="K63" s="6"/>
-      <c r="L63" s="6" t="s">
+      <c r="L63" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="M63" s="7"/>
-    </row>
-    <row r="64" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="M63" s="6"/>
+    </row>
+    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B64" s="5">
         <v>1006</v>
       </c>
-      <c r="C64" s="6"/>
-      <c r="D64" s="6" t="s">
+      <c r="D64" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E64" s="6"/>
-      <c r="F64" s="6">
+      <c r="F64" s="1">
         <v>1005</v>
       </c>
-      <c r="G64" s="6"/>
-      <c r="H64" s="6" t="s">
+      <c r="H64" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I64" s="6"/>
-      <c r="J64" s="6">
+      <c r="J64" s="1">
         <v>1006</v>
       </c>
-      <c r="K64" s="6"/>
-      <c r="L64" s="6" t="s">
+      <c r="L64" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M64" s="7"/>
+      <c r="M64" s="6"/>
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="5">
         <v>1007</v>
       </c>
-      <c r="C65" s="6"/>
-      <c r="D65" s="6" t="s">
+      <c r="D65" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E65" s="6"/>
-      <c r="F65" s="6">
+      <c r="F65" s="1">
         <v>1006</v>
       </c>
-      <c r="G65" s="6"/>
-      <c r="H65" s="6" t="s">
+      <c r="H65" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I65" s="6"/>
-      <c r="J65" s="6">
+      <c r="J65" s="1">
         <v>1007</v>
       </c>
-      <c r="K65" s="6"/>
-      <c r="L65" s="6" t="s">
+      <c r="L65" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="M65" s="7"/>
+      <c r="M65" s="6"/>
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B66" s="5">
         <v>1008</v>
       </c>
-      <c r="C66" s="6"/>
-      <c r="D66" s="6" t="s">
+      <c r="D66" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E66" s="6"/>
-      <c r="F66" s="6">
+      <c r="F66" s="1">
         <v>1008</v>
       </c>
-      <c r="G66" s="6"/>
-      <c r="H66" s="6" t="s">
+      <c r="H66" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I66" s="6"/>
-      <c r="J66" s="6">
+      <c r="J66" s="1">
         <v>1008</v>
       </c>
-      <c r="K66" s="6"/>
-      <c r="L66" s="6" t="s">
+      <c r="L66" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M66" s="7"/>
+      <c r="M66" s="6"/>
     </row>
     <row r="67" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B67" s="9" t="s">
+      <c r="B67" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C67" s="10"/>
-      <c r="D67" s="6"/>
-      <c r="E67" s="6"/>
-      <c r="F67" s="10" t="s">
+      <c r="C67" s="9"/>
+      <c r="F67" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G67" s="10"/>
-      <c r="H67" s="6"/>
-      <c r="I67" s="6"/>
-      <c r="J67" s="10" t="s">
+      <c r="G67" s="9"/>
+      <c r="J67" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="K67" s="10"/>
-      <c r="L67" s="6"/>
-      <c r="M67" s="7"/>
+      <c r="K67" s="9"/>
+      <c r="M67" s="6"/>
     </row>
     <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="5">
         <v>1098</v>
       </c>
-      <c r="C68" s="6"/>
-      <c r="D68" s="6" t="s">
+      <c r="D68" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E68" s="6"/>
-      <c r="F68" s="6">
+      <c r="F68" s="1">
         <v>1098</v>
       </c>
-      <c r="G68" s="6"/>
-      <c r="H68" s="6" t="s">
+      <c r="H68" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I68" s="6"/>
-      <c r="J68" s="6">
+      <c r="J68" s="1">
         <v>1098</v>
       </c>
-      <c r="K68" s="6"/>
-      <c r="L68" s="6" t="s">
+      <c r="L68" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M68" s="7"/>
+      <c r="M68" s="6"/>
     </row>
     <row r="69" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B69" s="12"/>
-      <c r="C69" s="13"/>
-      <c r="D69" s="13"/>
-      <c r="E69" s="13"/>
-      <c r="F69" s="13"/>
-      <c r="G69" s="13"/>
-      <c r="H69" s="13"/>
-      <c r="I69" s="13"/>
-      <c r="J69" s="13"/>
-      <c r="K69" s="13"/>
-      <c r="L69" s="13"/>
-      <c r="M69" s="14"/>
+      <c r="B69" s="11"/>
+      <c r="C69" s="12"/>
+      <c r="D69" s="12"/>
+      <c r="E69" s="12"/>
+      <c r="F69" s="12"/>
+      <c r="G69" s="12"/>
+      <c r="H69" s="12"/>
+      <c r="I69" s="12"/>
+      <c r="J69" s="12"/>
+      <c r="K69" s="12"/>
+      <c r="L69" s="12"/>
+      <c r="M69" s="13"/>
     </row>
     <row r="71" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="F71" s="6" t="s">
+      <c r="F71" s="1" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1998,256 +1665,203 @@
     </row>
     <row r="74" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B74" s="5"/>
-      <c r="C74" s="8" t="s">
+      <c r="C74" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D74" s="6"/>
-      <c r="E74" s="6"/>
-      <c r="F74" s="6"/>
-      <c r="G74" s="8" t="s">
+      <c r="G74" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H74" s="6"/>
-      <c r="I74" s="6"/>
-      <c r="J74" s="6"/>
-      <c r="K74" s="8" t="s">
+      <c r="K74" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L74" s="6"/>
-      <c r="M74" s="7"/>
+      <c r="M74" s="6"/>
     </row>
     <row r="75" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B75" s="5"/>
-      <c r="C75" s="6"/>
-      <c r="D75" s="6"/>
-      <c r="E75" s="6"/>
-      <c r="F75" s="6"/>
-      <c r="G75" s="6"/>
-      <c r="H75" s="6"/>
-      <c r="I75" s="6"/>
-      <c r="J75" s="6"/>
-      <c r="K75" s="6"/>
-      <c r="L75" s="6"/>
-      <c r="M75" s="7"/>
+      <c r="M75" s="6"/>
     </row>
     <row r="76" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B76" s="9" t="s">
+      <c r="B76" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C76" s="10"/>
-      <c r="D76" s="11" t="s">
+      <c r="C76" s="9"/>
+      <c r="D76" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E76" s="10"/>
-      <c r="F76" s="10" t="s">
+      <c r="E76" s="9"/>
+      <c r="F76" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="G76" s="10"/>
-      <c r="H76" s="11" t="s">
+      <c r="G76" s="9"/>
+      <c r="H76" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="I76" s="6"/>
-      <c r="J76" s="10" t="s">
+      <c r="J76" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="K76" s="10"/>
-      <c r="L76" s="6" t="s">
+      <c r="K76" s="9"/>
+      <c r="L76" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="M76" s="7"/>
+      <c r="M76" s="6"/>
     </row>
     <row r="77" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B77" s="5">
         <v>1001</v>
       </c>
-      <c r="C77" s="6"/>
-      <c r="D77" s="6" t="s">
+      <c r="D77" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E77" s="6"/>
-      <c r="F77" s="6">
+      <c r="F77" s="1">
         <v>1001</v>
       </c>
-      <c r="G77" s="6"/>
-      <c r="H77" s="6" t="s">
+      <c r="H77" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I77" s="6"/>
-      <c r="J77" s="6">
+      <c r="J77" s="1">
         <v>1001</v>
       </c>
-      <c r="K77" s="6"/>
-      <c r="L77" s="6" t="s">
+      <c r="L77" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M77" s="7"/>
+      <c r="M77" s="6"/>
     </row>
     <row r="78" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B78" s="5">
         <v>1002</v>
       </c>
-      <c r="C78" s="6"/>
-      <c r="D78" s="6" t="s">
+      <c r="D78" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E78" s="6"/>
-      <c r="F78" s="6">
+      <c r="F78" s="1">
         <v>1003</v>
       </c>
-      <c r="G78" s="6"/>
-      <c r="H78" s="6" t="s">
+      <c r="H78" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I78" s="6"/>
-      <c r="J78" s="6">
+      <c r="J78" s="1">
         <v>1003</v>
       </c>
-      <c r="K78" s="6"/>
-      <c r="L78" s="6" t="s">
+      <c r="L78" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="M78" s="7"/>
+      <c r="M78" s="6"/>
     </row>
     <row r="79" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B79" s="5">
         <v>1006</v>
       </c>
-      <c r="C79" s="6"/>
-      <c r="D79" s="6" t="s">
+      <c r="D79" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E79" s="6"/>
-      <c r="F79" s="6">
+      <c r="F79" s="1">
         <v>1005</v>
       </c>
-      <c r="G79" s="6"/>
-      <c r="H79" s="6" t="s">
+      <c r="H79" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I79" s="6"/>
-      <c r="J79" s="6">
+      <c r="J79" s="1">
         <v>1005</v>
       </c>
-      <c r="K79" s="6"/>
-      <c r="L79" s="6" t="s">
+      <c r="L79" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="M79" s="7"/>
+      <c r="M79" s="6"/>
     </row>
     <row r="80" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B80" s="5">
         <v>1007</v>
       </c>
-      <c r="C80" s="6"/>
-      <c r="D80" s="6" t="s">
+      <c r="D80" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E80" s="6"/>
-      <c r="F80" s="6">
+      <c r="F80" s="1">
         <v>1006</v>
       </c>
-      <c r="G80" s="6"/>
-      <c r="H80" s="6" t="s">
+      <c r="H80" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I80" s="6"/>
-      <c r="J80" s="6">
+      <c r="J80" s="1">
         <v>1006</v>
       </c>
-      <c r="K80" s="6"/>
-      <c r="L80" s="6" t="s">
+      <c r="L80" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M80" s="7"/>
+      <c r="M80" s="6"/>
     </row>
     <row r="81" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B81" s="5">
         <v>1008</v>
       </c>
-      <c r="C81" s="6"/>
-      <c r="D81" s="6" t="s">
+      <c r="D81" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E81" s="6"/>
-      <c r="F81" s="6">
+      <c r="F81" s="1">
         <v>1008</v>
       </c>
-      <c r="G81" s="6"/>
-      <c r="H81" s="6" t="s">
+      <c r="H81" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I81" s="6"/>
-      <c r="J81" s="6">
+      <c r="J81" s="1">
         <v>1008</v>
       </c>
-      <c r="K81" s="6"/>
-      <c r="L81" s="6" t="s">
+      <c r="L81" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M81" s="7"/>
+      <c r="M81" s="6"/>
     </row>
     <row r="82" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B82" s="9" t="s">
+      <c r="B82" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C82" s="10"/>
-      <c r="D82" s="6"/>
-      <c r="E82" s="6"/>
-      <c r="F82" s="10" t="s">
+      <c r="C82" s="9"/>
+      <c r="F82" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G82" s="10"/>
-      <c r="H82" s="6"/>
-      <c r="I82" s="6"/>
-      <c r="J82" s="10" t="s">
+      <c r="G82" s="9"/>
+      <c r="J82" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="K82" s="10"/>
-      <c r="L82" s="6"/>
-      <c r="M82" s="7"/>
+      <c r="K82" s="9"/>
+      <c r="M82" s="6"/>
     </row>
     <row r="83" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B83" s="5">
         <v>1098</v>
       </c>
-      <c r="C83" s="6"/>
-      <c r="D83" s="6" t="s">
+      <c r="D83" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E83" s="6"/>
-      <c r="F83" s="6">
+      <c r="F83" s="1">
         <v>1098</v>
       </c>
-      <c r="G83" s="6"/>
-      <c r="H83" s="6" t="s">
+      <c r="H83" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I83" s="6"/>
-      <c r="J83" s="6">
+      <c r="J83" s="1">
         <v>1098</v>
       </c>
-      <c r="K83" s="6"/>
-      <c r="L83" s="6" t="s">
+      <c r="L83" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M83" s="7"/>
+      <c r="M83" s="6"/>
     </row>
     <row r="84" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B84" s="12"/>
-      <c r="C84" s="13"/>
-      <c r="D84" s="13"/>
-      <c r="E84" s="13"/>
-      <c r="F84" s="13"/>
-      <c r="G84" s="13"/>
-      <c r="H84" s="13"/>
-      <c r="I84" s="13"/>
-      <c r="J84" s="13"/>
-      <c r="K84" s="13"/>
-      <c r="L84" s="13"/>
-      <c r="M84" s="14"/>
+      <c r="B84" s="11"/>
+      <c r="C84" s="12"/>
+      <c r="D84" s="12"/>
+      <c r="E84" s="12"/>
+      <c r="F84" s="12"/>
+      <c r="G84" s="12"/>
+      <c r="H84" s="12"/>
+      <c r="I84" s="12"/>
+      <c r="J84" s="12"/>
+      <c r="K84" s="12"/>
+      <c r="L84" s="12"/>
+      <c r="M84" s="13"/>
     </row>
     <row r="86" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="F86" s="6" t="s">
+      <c r="F86" s="1" t="s">
         <v>47</v>
       </c>
     </row>
@@ -2267,303 +1881,220 @@
     </row>
     <row r="89" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B89" s="5"/>
-      <c r="C89" s="8" t="s">
+      <c r="C89" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D89" s="6"/>
-      <c r="E89" s="6"/>
-      <c r="F89" s="6"/>
-      <c r="G89" s="8" t="s">
+      <c r="G89" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H89" s="6"/>
-      <c r="I89" s="6"/>
-      <c r="J89" s="6"/>
-      <c r="K89" s="8" t="s">
+      <c r="K89" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L89" s="6"/>
-      <c r="M89" s="7"/>
+      <c r="M89" s="6"/>
     </row>
     <row r="90" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B90" s="5"/>
-      <c r="C90" s="6"/>
-      <c r="D90" s="6"/>
-      <c r="E90" s="6"/>
-      <c r="F90" s="6"/>
-      <c r="G90" s="6"/>
-      <c r="H90" s="6"/>
-      <c r="I90" s="6"/>
-      <c r="J90" s="6"/>
-      <c r="K90" s="6"/>
-      <c r="L90" s="6"/>
-      <c r="M90" s="7"/>
+      <c r="M90" s="6"/>
     </row>
     <row r="91" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B91" s="9" t="s">
+      <c r="B91" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C91" s="10"/>
-      <c r="D91" s="11" t="s">
+      <c r="C91" s="9"/>
+      <c r="D91" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E91" s="10"/>
-      <c r="F91" s="10" t="s">
+      <c r="E91" s="9"/>
+      <c r="F91" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="G91" s="10"/>
-      <c r="H91" s="11" t="s">
+      <c r="G91" s="9"/>
+      <c r="H91" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="I91" s="6"/>
-      <c r="J91" s="10" t="s">
+      <c r="J91" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="K91" s="10"/>
-      <c r="L91" s="6" t="s">
+      <c r="K91" s="9"/>
+      <c r="L91" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="M91" s="7"/>
+      <c r="M91" s="6"/>
     </row>
     <row r="92" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B92" s="5">
         <v>1001</v>
       </c>
-      <c r="C92" s="6"/>
-      <c r="D92" s="6" t="s">
+      <c r="D92" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E92" s="6"/>
-      <c r="F92" s="6">
+      <c r="F92" s="1">
         <v>1001</v>
       </c>
-      <c r="G92" s="6"/>
-      <c r="H92" s="6" t="s">
+      <c r="H92" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I92" s="6"/>
-      <c r="J92" s="6">
+      <c r="J92" s="1">
         <v>1001</v>
       </c>
-      <c r="K92" s="6"/>
-      <c r="L92" s="6" t="s">
+      <c r="L92" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M92" s="7"/>
+      <c r="M92" s="6"/>
     </row>
     <row r="93" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B93" s="5">
         <v>1002</v>
       </c>
-      <c r="C93" s="6"/>
-      <c r="D93" s="6" t="s">
+      <c r="D93" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E93" s="6"/>
-      <c r="F93" s="6">
+      <c r="F93" s="1">
         <v>1003</v>
       </c>
-      <c r="G93" s="6"/>
-      <c r="H93" s="6" t="s">
+      <c r="H93" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I93" s="6"/>
-      <c r="J93" s="6">
+      <c r="J93" s="1">
         <v>1002</v>
       </c>
-      <c r="K93" s="6"/>
-      <c r="L93" s="6" t="s">
+      <c r="L93" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="M93" s="7"/>
+      <c r="M93" s="6"/>
     </row>
     <row r="94" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B94" s="5">
         <v>1006</v>
       </c>
-      <c r="C94" s="6"/>
-      <c r="D94" s="6" t="s">
+      <c r="D94" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E94" s="6"/>
-      <c r="F94" s="6">
+      <c r="F94" s="1">
         <v>1005</v>
       </c>
-      <c r="G94" s="6"/>
-      <c r="H94" s="6" t="s">
+      <c r="H94" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I94" s="6"/>
-      <c r="J94" s="6">
+      <c r="J94" s="1">
         <v>1003</v>
       </c>
-      <c r="K94" s="6"/>
-      <c r="L94" s="6" t="s">
+      <c r="L94" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="M94" s="7"/>
+      <c r="M94" s="6"/>
     </row>
     <row r="95" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B95" s="5">
         <v>1007</v>
       </c>
-      <c r="C95" s="6"/>
-      <c r="D95" s="6" t="s">
+      <c r="D95" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E95" s="6"/>
-      <c r="F95" s="6">
+      <c r="F95" s="1">
         <v>1006</v>
       </c>
-      <c r="G95" s="6"/>
-      <c r="H95" s="6" t="s">
+      <c r="H95" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I95" s="6"/>
-      <c r="J95" s="6">
+      <c r="J95" s="1">
         <v>1005</v>
       </c>
-      <c r="K95" s="6"/>
-      <c r="L95" s="6" t="s">
+      <c r="L95" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="M95" s="7"/>
+      <c r="M95" s="6"/>
     </row>
     <row r="96" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B96" s="5">
         <v>1008</v>
       </c>
-      <c r="C96" s="6"/>
-      <c r="D96" s="6" t="s">
+      <c r="D96" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E96" s="6"/>
-      <c r="F96" s="6">
+      <c r="F96" s="1">
         <v>1008</v>
       </c>
-      <c r="G96" s="6"/>
-      <c r="H96" s="6" t="s">
+      <c r="H96" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I96" s="6"/>
-      <c r="J96" s="6">
+      <c r="J96" s="1">
         <v>1006</v>
       </c>
-      <c r="K96" s="6"/>
-      <c r="L96" s="6" t="s">
+      <c r="L96" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M96" s="7"/>
+      <c r="M96" s="6"/>
     </row>
     <row r="97" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B97" s="9" t="s">
+      <c r="B97" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C97" s="10"/>
-      <c r="D97" s="6"/>
-      <c r="E97" s="6"/>
-      <c r="F97" s="10" t="s">
+      <c r="C97" s="9"/>
+      <c r="F97" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G97" s="10"/>
-      <c r="H97" s="6"/>
-      <c r="I97" s="6"/>
-      <c r="J97" s="6">
+      <c r="G97" s="9"/>
+      <c r="J97" s="1">
         <v>1007</v>
       </c>
-      <c r="K97" s="6"/>
-      <c r="L97" s="6" t="s">
+      <c r="L97" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="M97" s="7"/>
+      <c r="M97" s="6"/>
     </row>
     <row r="98" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B98" s="5">
         <v>1098</v>
       </c>
-      <c r="C98" s="6"/>
-      <c r="D98" s="6" t="s">
+      <c r="D98" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E98" s="6"/>
-      <c r="F98" s="6">
+      <c r="F98" s="1">
         <v>1098</v>
       </c>
-      <c r="G98" s="6"/>
-      <c r="H98" s="6" t="s">
+      <c r="H98" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I98" s="6"/>
-      <c r="J98" s="6">
+      <c r="J98" s="1">
         <v>1008</v>
       </c>
-      <c r="K98" s="6"/>
-      <c r="L98" s="6" t="s">
+      <c r="L98" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M98" s="7"/>
+      <c r="M98" s="6"/>
     </row>
     <row r="99" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B99" s="5"/>
-      <c r="C99" s="6"/>
-      <c r="D99" s="6"/>
-      <c r="E99" s="6"/>
-      <c r="F99" s="6"/>
-      <c r="G99" s="6"/>
-      <c r="H99" s="6"/>
-      <c r="I99" s="6"/>
-      <c r="J99" s="10" t="s">
+      <c r="J99" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="K99" s="10"/>
-      <c r="L99" s="6"/>
-      <c r="M99" s="7"/>
+      <c r="K99" s="9"/>
+      <c r="M99" s="6"/>
     </row>
     <row r="100" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B100" s="5"/>
-      <c r="C100" s="6"/>
-      <c r="D100" s="6"/>
-      <c r="E100" s="6"/>
-      <c r="F100" s="6"/>
-      <c r="G100" s="6"/>
-      <c r="H100" s="6"/>
-      <c r="I100" s="6"/>
-      <c r="J100" s="6">
+      <c r="J100" s="1">
         <v>1098</v>
       </c>
-      <c r="K100" s="6"/>
-      <c r="L100" s="6" t="s">
+      <c r="L100" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M100" s="7"/>
+      <c r="M100" s="6"/>
     </row>
     <row r="101" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B101" s="12"/>
-      <c r="C101" s="13"/>
-      <c r="D101" s="13"/>
-      <c r="E101" s="13"/>
-      <c r="F101" s="13"/>
-      <c r="G101" s="13"/>
-      <c r="H101" s="13"/>
-      <c r="I101" s="13"/>
-      <c r="J101" s="13"/>
-      <c r="K101" s="13"/>
-      <c r="L101" s="13"/>
-      <c r="M101" s="14"/>
-    </row>
-    <row r="102" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B102" s="6"/>
-      <c r="C102" s="6"/>
-      <c r="D102" s="6"/>
-      <c r="E102" s="6"/>
-      <c r="F102" s="6"/>
-      <c r="G102" s="6"/>
-      <c r="H102" s="6"/>
-      <c r="I102" s="6"/>
-      <c r="J102" s="6"/>
-      <c r="K102" s="6"/>
-      <c r="L102" s="6"/>
-      <c r="M102" s="6"/>
+      <c r="B101" s="11"/>
+      <c r="C101" s="12"/>
+      <c r="D101" s="12"/>
+      <c r="E101" s="12"/>
+      <c r="F101" s="12"/>
+      <c r="G101" s="12"/>
+      <c r="H101" s="12"/>
+      <c r="I101" s="12"/>
+      <c r="J101" s="12"/>
+      <c r="K101" s="12"/>
+      <c r="L101" s="12"/>
+      <c r="M101" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>